<commit_message>
Updated Excel test cases
</commit_message>
<xml_diff>
--- a/Practice Test Automation.xlsx
+++ b/Practice Test Automation.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="68">
   <si>
     <t>AI &amp; IT</t>
   </si>
@@ -105,18 +105,6 @@
     <t>Home_Button_Test.java</t>
   </si>
   <si>
-    <t>Home Button</t>
-  </si>
-  <si>
-    <t>Check Whether Home Page Open Correctly</t>
-  </si>
-  <si>
-    <t>Open Home Button and Check page Displayed</t>
-  </si>
-  <si>
-    <t>1)Open ChromeBrowser 2)Search practicetestautomation.com 3)Click Home Button 4)Check Result</t>
-  </si>
-  <si>
     <t>Pass</t>
   </si>
   <si>
@@ -127,18 +115,6 @@
   </si>
   <si>
     <t>Practice_Button_Test.java</t>
-  </si>
-  <si>
-    <t>Practice Button</t>
-  </si>
-  <si>
-    <t>Check Whether Practice Page Open Correctly</t>
-  </si>
-  <si>
-    <t>Open Practice Button and Check page Displayed</t>
-  </si>
-  <si>
-    <t>1)Open ChromeBrowser 2)Search practicetestautomation.com 3)Click Practice Button 4)Check Result</t>
   </si>
   <si>
     <r>
@@ -162,6 +138,150 @@
       </rPr>
       <t>:https://github.com/yogita20122006-netizen/Practice-Test-Automation</t>
     </r>
+  </si>
+  <si>
+    <t>3)</t>
+  </si>
+  <si>
+    <t>Courses_Link_Test.java</t>
+  </si>
+  <si>
+    <t>Course Link</t>
+  </si>
+  <si>
+    <t>Check Whether Course link Open Correctly</t>
+  </si>
+  <si>
+    <t>Open Course Link and Check Page Displayed</t>
+  </si>
+  <si>
+    <t>1)Open chromeBrowser 2)Search practicetestautomation.com 4)Click Course Link      5)Check Result</t>
+  </si>
+  <si>
+    <t>Practice Link</t>
+  </si>
+  <si>
+    <t>Home Link</t>
+  </si>
+  <si>
+    <t>Check Whether Home Link Open Correctly</t>
+  </si>
+  <si>
+    <t>Open Home Link and Check page Displayed</t>
+  </si>
+  <si>
+    <t>1)Open ChromeBrowser 2)Search practicetestautomation.com 3)Click Home link         4)Check Result</t>
+  </si>
+  <si>
+    <t>Check Whether Practice Link Open Correctly</t>
+  </si>
+  <si>
+    <t>Open Practice Link and Check page Displayed</t>
+  </si>
+  <si>
+    <t>1)Open ChromeBrowser 2)Search practicetestautomation.com 3)Click Practice Link 4)Check Result</t>
+  </si>
+  <si>
+    <t>4)</t>
+  </si>
+  <si>
+    <t>AIWORKSHOP_Link_Test.java</t>
+  </si>
+  <si>
+    <t>AI WORKSHOP Link</t>
+  </si>
+  <si>
+    <t>Check Whether AI WORKSHOP link Open Correctly</t>
+  </si>
+  <si>
+    <t>Open AI WORKSHOP link and Check Page Displayed</t>
+  </si>
+  <si>
+    <t>1)Open chromeBrowser 2)Search practicetestautomation.com 4)Click AI WORKSHOP Link      5)Check Result</t>
+  </si>
+  <si>
+    <t>5)</t>
+  </si>
+  <si>
+    <t>Blog_Link_Test.java</t>
+  </si>
+  <si>
+    <t>Blog Link</t>
+  </si>
+  <si>
+    <t>Check Whether Blog Link Open Correctly</t>
+  </si>
+  <si>
+    <t>Open Blog Link and Check page Displayed</t>
+  </si>
+  <si>
+    <t>1)Open chromeBrowser 2)Search practicetestautomation.com 4)Click BlogLink              5)Check Result</t>
+  </si>
+  <si>
+    <t>6)</t>
+  </si>
+  <si>
+    <t>Contact_Link_Test.java</t>
+  </si>
+  <si>
+    <t>Contact Link</t>
+  </si>
+  <si>
+    <t>1)Open chromeBrowser 2)Search practicetestautomation.com 4)Click ContactLink              5)Check Result</t>
+  </si>
+  <si>
+    <t>7)</t>
+  </si>
+  <si>
+    <t>Test_Exception_page_link.java</t>
+  </si>
+  <si>
+    <t>Test_login_page.java</t>
+  </si>
+  <si>
+    <t>Test Login page Link</t>
+  </si>
+  <si>
+    <t>Check Whether Test Login page Link in Practice Page Open Correctly</t>
+  </si>
+  <si>
+    <t>Open Test Login Page Link and Check page Displayed</t>
+  </si>
+  <si>
+    <t>1)Open chromeBrowser 2)Search practicetestautomation.com 4)Click Practice Link             5)Click Test login page link    6)Check Result</t>
+  </si>
+  <si>
+    <t>8)</t>
+  </si>
+  <si>
+    <t>Test Exceptions Link</t>
+  </si>
+  <si>
+    <t>Check Whether Test Exceptions Link in Practice Page Open Correctly</t>
+  </si>
+  <si>
+    <t>Open Test Exceptions Link and Check page Displayed</t>
+  </si>
+  <si>
+    <t>1)Open chromeBrowser 2)Search practicetestautomation.com 4)Click Practice Link             5)Click Test Exceptions link    6)Check Result</t>
+  </si>
+  <si>
+    <t>9)</t>
+  </si>
+  <si>
+    <t>Test_Table_link_Test.java</t>
+  </si>
+  <si>
+    <t>Test Table Link</t>
+  </si>
+  <si>
+    <t>Check Whether Test Table Link in Practice Page Open Correctly</t>
+  </si>
+  <si>
+    <t>Open Test TableLink and Check page Displayed</t>
+  </si>
+  <si>
+    <t>1)Open chromeBrowser 2)Search practicetestautomation.com 4)Click Practice Link             5)Click Test Table link    6)Check Result</t>
   </si>
 </sst>
 </file>
@@ -237,7 +357,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -268,6 +388,12 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -573,7 +699,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="14.28515625" style="2" customWidth="1"/>
@@ -627,7 +753,7 @@
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
       <c r="F4" s="9" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="G4" s="9"/>
       <c r="H4" s="9"/>
@@ -676,56 +802,190 @@
         <v>14</v>
       </c>
       <c r="C7" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="G7" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="H7" s="5" t="s">
         <v>16</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="H7" s="5" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="135.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="135.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="C9" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="D9" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="E9" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="F9" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="F8" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G8" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="H8" s="5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" ht="135.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="10" spans="1:9" ht="135.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="11" spans="1:9" ht="24.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="1:9" ht="24.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="13" spans="1:9" ht="24.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="14" spans="1:9" ht="24.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    </row>
+    <row r="10" spans="1:9" ht="135.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="127.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="125.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="D12" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="120.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="127.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="133.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>67</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A4:B5"/>

</xml_diff>